<commit_message>
Update Zoho import template to match user requirements
Update the CAS Zoho Import Template XLSX file to remove the Salutation column and rename the Institution column to "Institution (Company)" to align with Zoho CRM field naming conventions.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ef7bf022-0b3a-4156-9c38-2b98b837c1d1
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 68ef8c0a-2d37-48c7-b1dd-824d729bda99
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/e9fe007f-c11f-42ca-a1dd-347ccc032e17/ef7bf022-0b3a-4156-9c38-2b98b837c1d1/QF8c5Of
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/exports/CAS_Zoho_Import_Template.xlsx
+++ b/exports/CAS_Zoho_Import_Template.xlsx
@@ -399,32 +399,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:W1"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
     <col min="3" max="3" width="17.83203125" customWidth="1"/>
     <col min="4" max="4" width="19.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="28.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="28.83203125" customWidth="1"/>
+    <col min="5" max="5" width="28.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="25.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="28.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
     <col min="11" max="11" width="16.83203125" customWidth="1"/>
-    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="30.83203125" customWidth="1"/>
     <col min="13" max="13" width="30.83203125" customWidth="1"/>
-    <col min="14" max="14" width="30.83203125" customWidth="1"/>
-    <col min="15" max="15" width="26.83203125" customWidth="1"/>
-    <col min="16" max="16" width="19.83203125" customWidth="1"/>
+    <col min="14" max="14" width="26.83203125" customWidth="1"/>
+    <col min="15" max="15" width="19.83203125" customWidth="1"/>
+    <col min="16" max="16" width="16.83203125" customWidth="1"/>
     <col min="17" max="17" width="16.83203125" customWidth="1"/>
     <col min="18" max="18" width="16.83203125" customWidth="1"/>
-    <col min="19" max="19" width="16.83203125" customWidth="1"/>
-    <col min="20" max="20" width="19.83203125" customWidth="1"/>
-    <col min="21" max="21" width="20.83203125" customWidth="1"/>
-    <col min="22" max="22" width="18.83203125" customWidth="1"/>
-    <col min="23" max="23" width="23.83203125" customWidth="1"/>
-    <col min="24" max="24" width="24.83203125" customWidth="1"/>
+    <col min="19" max="19" width="19.83203125" customWidth="1"/>
+    <col min="20" max="20" width="20.83203125" customWidth="1"/>
+    <col min="21" max="21" width="18.83203125" customWidth="1"/>
+    <col min="22" max="22" width="23.83203125" customWidth="1"/>
+    <col min="23" max="23" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -441,76 +440,73 @@
         <v>Secondary Email</v>
       </c>
       <c r="E1" t="str">
-        <v>Salutation</v>
+        <v>Professional Designation</v>
       </c>
       <c r="F1" t="str">
-        <v>Professional Designation</v>
+        <v>Subspecialty</v>
       </c>
       <c r="G1" t="str">
-        <v>Subspecialty</v>
+        <v>Institution (Company)</v>
       </c>
       <c r="H1" t="str">
-        <v>Institution</v>
+        <v>Amyloidosis Type</v>
       </c>
       <c r="I1" t="str">
-        <v>Amyloidosis Type</v>
+        <v>Amyloidosis Type - Other</v>
       </c>
       <c r="J1" t="str">
-        <v>Amyloidosis Type - Other</v>
+        <v>CAS Member</v>
       </c>
       <c r="K1" t="str">
-        <v>CAS Member</v>
+        <v>CANN Member</v>
       </c>
       <c r="L1" t="str">
-        <v>CANN Member</v>
+        <v>CAS Communications Consent</v>
       </c>
       <c r="M1" t="str">
-        <v>CAS Communications Consent</v>
+        <v>CANN Communications Consent</v>
       </c>
       <c r="N1" t="str">
-        <v>CANN Communications Consent</v>
+        <v>Services Map Inclusion</v>
       </c>
       <c r="O1" t="str">
-        <v>Services Map Inclusion</v>
+        <v>Map Clinic Name</v>
       </c>
       <c r="P1" t="str">
-        <v>Map Clinic Name</v>
+        <v>Map Street</v>
       </c>
       <c r="Q1" t="str">
-        <v>Map Street</v>
+        <v>Map City</v>
       </c>
       <c r="R1" t="str">
-        <v>Map City</v>
+        <v>Map Province</v>
       </c>
       <c r="S1" t="str">
-        <v>Map Province</v>
+        <v>Map Postal Code</v>
       </c>
       <c r="T1" t="str">
-        <v>Map Postal Code</v>
+        <v>Map Clinic Phone</v>
       </c>
       <c r="U1" t="str">
-        <v>Map Clinic Phone</v>
+        <v>Map Clinic Fax</v>
       </c>
       <c r="V1" t="str">
-        <v>Map Clinic Fax</v>
+        <v>Description / Notes</v>
       </c>
       <c r="W1" t="str">
-        <v>Description / Notes</v>
-      </c>
-      <c r="X1" t="str">
         <v>Form Submission Date</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:X1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D24"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -590,91 +586,91 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Salutation</v>
+        <v>Professional Designation</v>
       </c>
       <c r="B6" t="str">
-        <v>Optional</v>
+        <v>Required for members</v>
       </c>
       <c r="C6" t="str">
-        <v>Dr., Prof., Mr., Mrs., Ms., Mx.</v>
+        <v>Free text (e.g., Cardiology, Hematology, Neurology, Nephrology)</v>
       </c>
       <c r="D6" t="str">
-        <v>Title. The live form no longer asks this, but you can set it for imported records.</v>
+        <v>The person's discipline. -&gt; Zoho 'Professional Designation'.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Professional Designation</v>
+        <v>Subspecialty</v>
       </c>
       <c r="B7" t="str">
         <v>Required for members</v>
       </c>
       <c r="C7" t="str">
-        <v>Free text (e.g., Cardiology, Hematology, Neurology, Nephrology)</v>
+        <v>Free text</v>
       </c>
       <c r="D7" t="str">
-        <v>The person's discipline. -&gt; Zoho 'Professional Designation'.</v>
+        <v>Sub-specialty area. -&gt; Zoho 'subspecialty'.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Subspecialty</v>
+        <v>Institution (Company)</v>
       </c>
       <c r="B8" t="str">
-        <v>Required for members</v>
+        <v>Optional</v>
       </c>
       <c r="C8" t="str">
         <v>Free text</v>
       </c>
       <c r="D8" t="str">
-        <v>Sub-specialty area. -&gt; Zoho 'subspecialty'.</v>
+        <v>Clinic / centre / hospital name. -&gt; Zoho 'Institution (Company)'.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Institution</v>
+        <v>Amyloidosis Type</v>
       </c>
       <c r="B9" t="str">
-        <v>Optional</v>
+        <v>Required for members</v>
       </c>
       <c r="C9" t="str">
-        <v>Free text</v>
+        <v>ATTR | AL | Both ATTR and AL | Other</v>
       </c>
       <c r="D9" t="str">
-        <v>Clinic / centre / hospital name. -&gt; Zoho 'Company'.</v>
+        <v>Pick ONE exactly as written. If 'Other', fill the next column.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Amyloidosis Type</v>
+        <v>Amyloidosis Type - Other</v>
       </c>
       <c r="B10" t="str">
-        <v>Required for members</v>
+        <v>Required only if Type = Other</v>
       </c>
       <c r="C10" t="str">
-        <v>ATTR | AL | Both ATTR and AL | Other</v>
+        <v>Free text</v>
       </c>
       <c r="D10" t="str">
-        <v>Pick ONE exactly as written. If 'Other', fill the next column.</v>
+        <v>The specific type when Amyloidosis Type is 'Other'. -&gt; Zoho 'Amyloidosis_Type_Other'.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Amyloidosis Type - Other</v>
+        <v>CAS Member</v>
       </c>
       <c r="B11" t="str">
-        <v>Required only if Type = Other</v>
+        <v>Required</v>
       </c>
       <c r="C11" t="str">
-        <v>Free text</v>
+        <v>Yes | No</v>
       </c>
       <c r="D11" t="str">
-        <v>The specific type when Amyloidosis Type is 'Other'. -&gt; Zoho 'Amyloidosis_Type_Other'.</v>
+        <v>Is this person a CAS member? NOTE: if CANN Member = Yes, this is automatically forced to Yes.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>CAS Member</v>
+        <v>CANN Member</v>
       </c>
       <c r="B12" t="str">
         <v>Required</v>
@@ -683,26 +679,26 @@
         <v>Yes | No</v>
       </c>
       <c r="D12" t="str">
-        <v>Is this person a CAS member? NOTE: if CANN Member = Yes, this is automatically forced to Yes.</v>
+        <v>Is this person a CANN member?</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>CANN Member</v>
+        <v>CAS Communications Consent</v>
       </c>
       <c r="B13" t="str">
-        <v>Required</v>
+        <v>Optional</v>
       </c>
       <c r="C13" t="str">
         <v>Yes | No</v>
       </c>
       <c r="D13" t="str">
-        <v>Is this person a CANN member?</v>
+        <v>Did they opt in to CAS emails? -&gt; Zoho 'CAS_Communications'.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>CAS Communications Consent</v>
+        <v>CANN Communications Consent</v>
       </c>
       <c r="B14" t="str">
         <v>Optional</v>
@@ -711,12 +707,12 @@
         <v>Yes | No</v>
       </c>
       <c r="D14" t="str">
-        <v>Did they opt in to CAS emails? -&gt; Zoho 'CAS_Communications'.</v>
+        <v>Did they opt in to CANN emails? -&gt; Zoho 'CANN_Communications'.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>CANN Communications Consent</v>
+        <v>Services Map Inclusion</v>
       </c>
       <c r="B15" t="str">
         <v>Optional</v>
@@ -725,26 +721,26 @@
         <v>Yes | No</v>
       </c>
       <c r="D15" t="str">
-        <v>Did they opt in to CANN emails? -&gt; Zoho 'CANN_Communications'.</v>
+        <v>Include their clinic on the public services map? If 'No', leave the 7 Map columns blank.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Services Map Inclusion</v>
+        <v>Map Clinic Name</v>
       </c>
       <c r="B16" t="str">
-        <v>Optional</v>
+        <v>Only if Map = Yes</v>
       </c>
       <c r="C16" t="str">
-        <v>Yes | No</v>
+        <v>Free text</v>
       </c>
       <c r="D16" t="str">
-        <v>Include their clinic on the public services map? If 'No', leave the 7 Map columns blank.</v>
+        <v>Clinic/centre name to show on the map. -&gt; Zoho 'Map_Clinic_Name'.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Map Clinic Name</v>
+        <v>Map Street</v>
       </c>
       <c r="B17" t="str">
         <v>Only if Map = Yes</v>
@@ -753,12 +749,12 @@
         <v>Free text</v>
       </c>
       <c r="D17" t="str">
-        <v>Clinic/centre name to show on the map. -&gt; Zoho 'Map_Clinic_Name'.</v>
+        <v>Street address. -&gt; Zoho 'Map_Street'.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Map Street</v>
+        <v>Map City</v>
       </c>
       <c r="B18" t="str">
         <v>Only if Map = Yes</v>
@@ -767,110 +763,96 @@
         <v>Free text</v>
       </c>
       <c r="D18" t="str">
-        <v>Street address. -&gt; Zoho 'Map_Street'.</v>
+        <v>City. -&gt; Zoho 'Map_City'.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Map City</v>
+        <v>Map Province</v>
       </c>
       <c r="B19" t="str">
         <v>Only if Map = Yes</v>
       </c>
       <c r="C19" t="str">
-        <v>Free text</v>
+        <v>Alberta | British Columbia | Manitoba | New Brunswick | Newfoundland and Labrador | Northwest Territories | Nova Scotia | Nunavut | Ontario | Prince Edward Island | Quebec | Saskatchewan | Yukon</v>
       </c>
       <c r="D19" t="str">
-        <v>City. -&gt; Zoho 'Map_City'.</v>
+        <v>Full province name, spelled exactly. -&gt; Zoho 'Map_Province'.</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Map Province</v>
+        <v>Map Postal Code</v>
       </c>
       <c r="B20" t="str">
         <v>Only if Map = Yes</v>
       </c>
       <c r="C20" t="str">
-        <v>Alberta | British Columbia | Manitoba | New Brunswick | Newfoundland and Labrador | Northwest Territories | Nova Scotia | Nunavut | Ontario | Prince Edward Island | Quebec | Saskatchewan | Yukon</v>
+        <v>Canadian postal code (e.g., M5H 2N2)</v>
       </c>
       <c r="D20" t="str">
-        <v>Full province name, spelled exactly. -&gt; Zoho 'Map_Province'.</v>
+        <v>Auto-uppercased on import. -&gt; Zoho 'Map_Postal_Code'.</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Map Postal Code</v>
+        <v>Map Clinic Phone</v>
       </c>
       <c r="B21" t="str">
         <v>Only if Map = Yes</v>
       </c>
       <c r="C21" t="str">
-        <v>Canadian postal code (e.g., M5H 2N2)</v>
+        <v>10 digits incl. area code</v>
       </c>
       <c r="D21" t="str">
-        <v>Auto-uppercased on import. -&gt; Zoho 'Map_Postal_Code'.</v>
+        <v>-&gt; Zoho 'Map_Clinic_Phone'.</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Map Clinic Phone</v>
+        <v>Map Clinic Fax</v>
       </c>
       <c r="B22" t="str">
-        <v>Only if Map = Yes</v>
+        <v>Optional (Map = Yes)</v>
       </c>
       <c r="C22" t="str">
         <v>10 digits incl. area code</v>
       </c>
       <c r="D22" t="str">
-        <v>-&gt; Zoho 'Map_Clinic_Phone'.</v>
+        <v>-&gt; Zoho 'Map_Clinic_Fax'.</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Map Clinic Fax</v>
+        <v>Description / Notes</v>
       </c>
       <c r="B23" t="str">
-        <v>Optional (Map = Yes)</v>
+        <v>Optional</v>
       </c>
       <c r="C23" t="str">
-        <v>10 digits incl. area code</v>
+        <v>Free text</v>
       </c>
       <c r="D23" t="str">
-        <v>-&gt; Zoho 'Map_Clinic_Fax'.</v>
+        <v>Inquiry message or any notes. -&gt; Zoho 'Description'. Mainly for non-members.</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Description / Notes</v>
+        <v>Form Submission Date</v>
       </c>
       <c r="B24" t="str">
         <v>Optional</v>
       </c>
       <c r="C24" t="str">
-        <v>Free text</v>
+        <v>YYYY-MM-DD or full date</v>
       </c>
       <c r="D24" t="str">
-        <v>Inquiry message or any notes. -&gt; Zoho 'Description'. Mainly for non-members.</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>Form Submission Date</v>
-      </c>
-      <c r="B25" t="str">
-        <v>Optional</v>
-      </c>
-      <c r="C25" t="str">
-        <v>YYYY-MM-DD or full date</v>
-      </c>
-      <c r="D25" t="str">
         <v>When they originally signed up. If blank, import time is used. -&gt; Zoho 'Form_Submission_Date'.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D24"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -949,7 +931,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v xml:space="preserve">  - Member rows: fill First Name, Last Name, Primary Email, Professional Designation, Subspecialty, Amyloidosis Type, Institution.</v>
+        <v xml:space="preserve">  - Member rows: fill First Name, Last Name, Primary Email, Professional Designation, Subspecialty, Amyloidosis Type, Institution (Company).</v>
       </c>
     </row>
     <row r="15">

</xml_diff>